<commit_message>
feat(ui): add modern Light Theme matching marketing_parameter CRM aesthetic and improve dashboard bridge
</commit_message>
<xml_diff>
--- a/data/verified_step1/step1_verified_dogs_latest.xlsx
+++ b/data/verified_step1/step1_verified_dogs_latest.xlsx
@@ -428,17 +428,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -495,36 +495,1838 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>61579338393951</t>
+          <t>100081804938692</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>mazora</t>
+          <t>Redhill Boykin Spaniels</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61579338393951</t>
+          <t>https://www.facebook.com/RedhillBoykinSpaniels</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Cún cưng đạt chuẩn AI Thị Giác (P_dog=0.82)</t>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: boykin, spaniels)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>adult_dog (P=0.82)</t>
+          <t>non_dog (P=0.85)</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.8197</v>
-      </c>
-      <c r="H2" t="inlineStr"/>
+        <v>0.85</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>boykin, spaniels</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn2-4.fna.fbcdn.net/v/t39.30808-1/759871619_122169590066977946_1033339009703974655_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx736x743&amp;ctp=p80x80&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=edfymLxSlhcQ7kNvwGo_utM&amp;_nc_oc=AdqayCmQ7nC2NpGSO9ex1Wyhrr5K_kEpivoHEmG_aszu5kPYlUqVpl-IawGgowKzqec&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-4.fna&amp;_nc_gid=SWF0arEU3Hh5DrS2xgAVSQ&amp;_nc_ss=7b2a8&amp;oh=00_AQOo25OoOPF8iCLA_l1pu1blSev83dZoujlskE1Rq201nw&amp;oe=6ADB8071</t>
+          <t>https://scontent.fsgn2-10.fna.fbcdn.net/v/t39.30808-1/780104405_1042413175162171_4016551396372726401_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=jL82okdLHuoQ7kNvwG407i7&amp;_nc_oc=AdoueWHs-w3xyO8dxkD01gpGC24aZuBmuD_qIwoa7cZe-jWTAyMWAoqbGB3zLT-AFq0&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-10.fna&amp;_nc_gid=j0SeNJfMMuxlZ_D87eT2sw&amp;_nc_ss=7b2a8&amp;oh=00_AQPiLtZZxwXSdcH6Psq_ROhy73414EKsDDtCsOTtmyK0Rw&amp;oe=6ADBE33E</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>61552753361052</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Eliana’s Shih Tzu Home</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61552753361052</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: shih tzu, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>shih tzu</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-4.fna.fbcdn.net/v/t39.30808-1/838967521_122256247310091778_3876985609640057852_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1320x1320&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=SqzPzn63QhcQ7kNvwFLcTW7&amp;_nc_oc=Ador46L1zHe8l3A2JTGrIxwI7_EOQIrtFWNjYxDI1kX9F-1RgNVtONrOKQeURDKXU8s&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-4.fna&amp;_nc_gid=j0SeNJfMMuxlZ_D87eT2sw&amp;_nc_ss=7b2a8&amp;oh=00_AQPiuEKdWhlMJW8xACgF9C3gRtHIAXr_FoG-x7b5vk9p-g&amp;oe=6ADBC2A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>100068177232065</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Family Loved Golden Retrievers</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/FamilyLovedGoldenRetrievers</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: golden retrievers, retrievers, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>golden retrievers, retrievers, goldens</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-10.fna.fbcdn.net/v/t39.30808-1/326488783_909141020535285_7958935178343501974_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=D_B4l-l7Tr4Q7kNvwHKjELe&amp;_nc_oc=AdoNU-z88TOi00VA6AS6n6QexAOKCyQoETgBH4NIOubc8eydMfJzzmW62GCRS29uEBk&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-10.fna&amp;_nc_gid=j0SeNJfMMuxlZ_D87eT2sw&amp;_nc_ss=7b2a8&amp;oh=00_AQN1srU1G6SeyBAl7CcmUOJ70PbXmI4eHXnFxCKe5L2kvw&amp;oe=6ADBB2C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>61591593760286</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>I Love Dogs Forge 'N Fetch</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61591593760286</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dogs, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>puppy (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>dogs</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-9.fna.fbcdn.net/v/t39.30808-1/753954046_122112615273386458_4146374115223244916_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1079x1078&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Ni6iO7UEIhAQ7kNvwGHxjBt&amp;_nc_oc=AdpMIU3a5raFnQaDZiQSnTecMLIM1v8IvA_g2uV78ELnJCybO5lk1fnqtDO4jX2gBOs&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-9.fna&amp;_nc_gid=j0SeNJfMMuxlZ_D87eT2sw&amp;_nc_ss=7b2a8&amp;oh=00_AQOlZZCosOXFbJljb0KBckpIsMHMw9LWZ3SCz_cVgNww0A&amp;oe=6ADBD84D</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>61594775080228</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yorkshih Pupco</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61594775080228</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: breeder, breeders, pupco)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.95)</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>breeder, breeders, pupco, yorkshire, shih tzu, pup, puppy, dog</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-11.fna.fbcdn.net/v/t39.30808-1/830513831_122102418099492502_4902222354387580447_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx800x800&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=yqqkmQ3XwqwQ7kNvwHAA1L2&amp;_nc_oc=AdqqiGgrByYtjyEA-9XGq5_zCmRQdGgY-61-mXsCSjxNsYcvtO5rG6AIjGR-jQsSVkE&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-11.fna&amp;_nc_gid=j0SeNJfMMuxlZ_D87eT2sw&amp;_nc_ss=7b2a8&amp;oh=00_AQPwvObvzfopmKxAynjQH3FGITqj-UP5rFSPaUtbdaPSNA&amp;oe=6ADBDCF5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>61551532070511</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Oakhaven Acres Aussies- AKC Australian Shepherds</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61551532070511</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: akc, shepherds, aussies)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.95)</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>akc, shepherds, aussies, australian shepherd</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-9.fna.fbcdn.net/v/t39.30808-1/427143042_122133778058051069_7335697382670797595_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1170x1170&amp;_nc_cat=102&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=S1XDbXl9UtEQ7kNvwF4VIVk&amp;_nc_oc=AdpxD3TijcgH-ylSuL5NrmZ1p7yt14Kbwa6RufX4zIILnneKdKQceOn1El-5DkI80-I&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-9.fna&amp;_nc_gid=8Zyh4tKsMAoxt1Skryj7PA&amp;_nc_ss=7b2a8&amp;oh=00_AQOxub4NnJJATL-nY2He740qF4xjBGX_kDJcZWkpFTnpZg&amp;oe=6ADBCAD2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>61588242310496</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Bottom Top Basset’s</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61588242310496</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: basset)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>basset</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-4.fna.fbcdn.net/v/t39.30808-1/825267903_122124942699274743_5172081817443253017_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=GKU7JoN128cQ7kNvwEAg_tV&amp;_nc_oc=Adp5wK-iRPL1nGSeTn3nSouGZKT-77wKX2f-GEt4J23kePf3pnnIMZYPzllcl12NlwQ&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-4.fna&amp;_nc_gid=8Zyh4tKsMAoxt1Skryj7PA&amp;_nc_ss=7b2a8&amp;oh=00_AQPfmOc7-4IEABA8EDi5ExLNh7hEjY3Wn5wlgmCDJPOcyg&amp;oe=6ADBE851</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>61594781858150</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Pawsome Daschund Puppies</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61594781858150</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, puppy, dog)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>puppies, puppy, dog</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-9.fna.fbcdn.net/v/t39.30808-1/839806917_122108759649492728_2289165301397021762_n.jpg?stp=c0.0.540.540a_cp0_dst-jpg_tt6&amp;cstp=mx540x540&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=UhsWya0bu5kQ7kNvwG_217d&amp;_nc_oc=Adqk7RM_dAOkyv9q40RlVNemofbyvYp40K5XZJzyvGfPv7pNhL0PWXtbXJsJTKEA5t4&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-9.fna&amp;_nc_gid=9RXVtVSJcH_YehD813TmiA&amp;_nc_ss=7b2a8&amp;oh=00_AQP6GAqyoklUO7MNX7_KuRevmML6Wq4mxYpkgdBB5nY4Tg&amp;oe=6ADBCC40</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>100063674375803</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tambali Pembroke welsh corgis est. 1998</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Tambalicorgis</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: corgis, pembroke)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>corgis, pembroke</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-3.fna.fbcdn.net/v/t39.30808-1/628787013_1489668089832323_6013872381075739493_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1024x1024&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=78QAEnU19pYQ7kNvwGxYj8E&amp;_nc_oc=Adp1_ysIFfL_ILZmD1llcOAqAgQGpRh8-bu01Ugxw-mGRYxzUHPuROdFO-cMG6KK7Zk&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-3.fna&amp;_nc_gid=Zn6-z2pa6UnZwcMXwHj8pA&amp;_nc_ss=7b2a8&amp;oh=00_AQOqV8enGX20V0zZIYxfibxiUdMiQxfSOouiFAmfVpZq1Q&amp;oe=6ADBD927</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>61591427093472</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Franklineschipperkes Kennel</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61591427093472</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: kennel)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>kennel</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-8.fna.fbcdn.net/v/t39.30808-1/818936768_122125355133380903_6137241591030814058_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx845x845&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=hekGuXarAzkQ7kNvwFVhA0T&amp;_nc_oc=AdrhXQuZ2r2xWnXzPuaitY67ho4W1Uu2P0H-ChBUbnSTnlsjI6ZGXACi3GdXfBFuvw8&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-8.fna&amp;_nc_gid=Zn6-z2pa6UnZwcMXwHj8pA&amp;_nc_ss=7b2a8&amp;oh=00_AQPDZrF7f3U2GHRvEFi7VhQta_FphM2zl9sbwsoy6U9TuQ&amp;oe=6ADBDC59</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>61593315111061</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Dachshund Puppies For Adoption And Rehoming</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61593315111061</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, dachshund, puppy)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>puppy (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>puppies, dachshund, puppy, dog</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-4.fna.fbcdn.net/v/t39.30808-1/766890471_122093395911443837_496170756872224230_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx828x828&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=_khz97jsH30Q7kNvwEoZtd2&amp;_nc_oc=Ado0UpHZ06X4SiSL-zc9nhg5xJnYqeeKKk-KojS8mp0AZQZTVWTWzQrr86RZqRoPgmQ&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-4.fna&amp;_nc_gid=Zn6-z2pa6UnZwcMXwHj8pA&amp;_nc_ss=7b2a8&amp;oh=00_AQNtKwvo2HswAU6FKyem4e4JCb1bUvVekZH280ZSBOFFMQ&amp;oe=6ADBC14E</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>61594494459425</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Autumn's Aussies</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61594494459425</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: aussies, australian shepherd, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>puppy (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>aussies, australian shepherd</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-5.fna.fbcdn.net/v/t39.30808-1/820934527_2313498826091469_1498160885209143484_n.jpg?stp=c0.0.1536.1536a_cp0_dst-jpg_tt6&amp;cstp=mx1536x1536&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=5q-lLkTmkTgQ7kNvwGzlRsF&amp;_nc_oc=AdqpEePssaVnFqEWRqbIEjIOE91zoirz9ecUMgad6Nnvu3KYJLkjCKkA9yal-kdBxm8&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-5.fna&amp;_nc_gid=uxKwerkAu71oeJTU8diDNw&amp;_nc_ss=7b2a8&amp;oh=00_AQPVTpjZHmNj0QRRQNRedJtciHiCo-DxBtcS1hTKbOPChA&amp;oe=6ADBD529</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>100040041254193</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pelican &amp; Friends</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Pelican.and.friends</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>AI Thị giác nhận diện chó trưởng thành (Adult=0.92, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>0.9982</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-11.fna.fbcdn.net/v/t39.30808-1/292449699_737020464309322_6439185362993122046_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x959&amp;_nc_cat=102&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=LTSee7h_BCcQ7kNvwEsNRrO&amp;_nc_oc=AdrCb02kFEvmuIRIQOTUp0S6qkXZtwBZO4HukxPIxGAkOxKLtokQhVQhS3XEfy08hiU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-11.fna&amp;_nc_gid=uxKwerkAu71oeJTU8diDNw&amp;_nc_ss=7b2a8&amp;oh=00_AQO28pmefPePozwXzomO3STNAAH-xMX3IiGsHAgRIKOdMg&amp;oe=6ADBB8F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>61568326866118</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Knock &amp; Bark Miniature Schnauzer.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/knockandbark</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: schnauzer, miniature schnauzer, P_dog=0.97)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>puppy (P=0.97)</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>0.9741</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>schnauzer, miniature schnauzer</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-9.fna.fbcdn.net/v/t39.30808-1/779082815_122193681896610895_1254854747032187011_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1134x1122&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=N6pIjA1Ts40Q7kNvwGoXvFJ&amp;_nc_oc=AdrsvN9GYTA_JFSxb7DGQJu8Dv8YGt5E3brZ6TW9oCZANRmnCWIJo2Ir1xaQh61ChtY&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-9.fna&amp;_nc_gid=uxKwerkAu71oeJTU8diDNw&amp;_nc_ss=7b2a8&amp;oh=00_AQO1sv4XiQKg9d9I8Jc40FaE9WsQLQUKMuQMYzaAMyrr0w&amp;oe=6ADBC47C</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>61593913773814</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Responsible Breeder Mentorship Program</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61593913773814</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: breeder)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.95)</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>breeder</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-8.fna.fbcdn.net/v/t39.30808-1/789960755_10215640356039617_8106197547239706512_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=zzjq-DH2fe4Q7kNvwGHGEwa&amp;_nc_oc=Ado-2hwNBIorQIVT9zd-qzC17gfV6ucydKQFaS0Ok5nOZ2auysfW0f9_XGOVRoDcV5w&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-8.fna&amp;_nc_gid=uxKwerkAu71oeJTU8diDNw&amp;_nc_ss=7b2a8&amp;oh=00_AQMcdWDNw9S4H3nuk3LCxVUC7AKzKyvpwgZ7R1jL0Vh8zw&amp;oe=6ADBC6C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>61551260240234</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>948 Cane Corso</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61551260240234</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: cane corso, corso)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>cane corso, corso</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-6.fna.fbcdn.net/v/t39.30808-1/405246072_122127983492042008_5422575660859054780_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1448x1448&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=1SHxRRdZeYcQ7kNvwGamyVp&amp;_nc_oc=AdptNJkAUw0hm7cNyVcCHwz4JCN5KhMk5Onivcd7bz9KgME_VP4iM0UeGpdZNHUg14I&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-6.fna&amp;_nc_gid=uxKwerkAu71oeJTU8diDNw&amp;_nc_ss=7b2a8&amp;oh=00_AQNkuYNPVt2P1CVbMEOs-qV_a8eoATd1quGKFLpeGaGvkw&amp;oe=6ADBE2AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>61594727570399</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Polly's Farm Pembroke Welsh Corgis &amp; Miniature Dachshunds</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61594727570399</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: corgis, pembroke, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>corgis, pembroke, dachshunds</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-8.fna.fbcdn.net/v/t39.30808-1/816996336_122112476091444595_648359482195584616_n.jpg?stp=c0.0.1220.1220a_cp0_dst-jpg_tt6&amp;cstp=mx1220x1220&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=jNFPSRSVDEMQ7kNvwFaeJes&amp;_nc_oc=AdrNnh_HCpL2LlpuavPbPhukTb6SAOcebtPTO69RzSrJLmwDFfrTbAoo5ybzxKn2B_Y&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-8.fna&amp;_nc_gid=uxKwerkAu71oeJTU8diDNw&amp;_nc_ss=7b2a8&amp;oh=00_AQMRZMoMteOvJgjV4ojJJYmzl0rqMWxmRfQlOAXvCSWlCw&amp;oe=6ADBD537</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>61594358583267</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>The Daily Doggo</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61594358583267</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: dog)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>dog</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-8.fna.fbcdn.net/v/t39.30808-1/805763280_10176161854575422_4288387135773466042_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1024x1024&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=wJuGISXnO18Q7kNvwHlv8XJ&amp;_nc_oc=AdrZzh17CyEkwDOZ-X1POoBJhW6O122k1ByheNBnUTm8P51m9HFyETAr2vpvfdO7zo4&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-8.fna&amp;_nc_gid=uxKwerkAu71oeJTU8diDNw&amp;_nc_ss=7b2a8&amp;oh=00_AQMGuC7Ym2NbNkjZRFZ4imuJghav05ktPwMLB45l_CKs-w&amp;oe=6ADBB274</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>61594354922562</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Linda Rottweiler puppy for adoption</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61594354922562</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppy, rottweiler, dog)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>puppy, rottweiler, dog</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-5.fna.fbcdn.net/v/t39.30808-1/843551321_122120349219478497_6210589935705443458_n.jpg?stp=c0.0.720.720a_cp0_dst-jpg_tt6&amp;cstp=mx720x720&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=wIsUI-6JU8UQ7kNvwHqqZvz&amp;_nc_oc=Adom3NuRjs_KsSAB5Hewt6k85k7onmSOhhK7zhVY3nKo6XJq-t7S70K1DYWStHAWaoI&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-5.fna&amp;_nc_gid=T8OyLSbfD_RUaywOpxI1wg&amp;_nc_ss=7b2a8&amp;oh=00_AQPbPZ0-GCR1s3L5gG8znUOkuc6tVtcdkAHZ-HU-iEtipg&amp;oe=6ADBBFAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>61594523153572</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Heartland Schnauzer Puppies for Adoption &amp; Rehoming</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61594523153572</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, schnauzer, puppy)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>puppy (P=0.95)</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>puppies, schnauzer, puppy, dog</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-6.fna.fbcdn.net/v/t39.30808-1/810246531_122095004037484105_2142050790308638206_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1199x1208&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=UghD7V6oAswQ7kNvwGB-qMd&amp;_nc_oc=AdpsFmmR4TXTBkjAPwOOww3yg-jpuff3qEJXSa4EWzeOhsGPQb2ZZcfK4zhhO0CGF6E&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-6.fna&amp;_nc_gid=T8OyLSbfD_RUaywOpxI1wg&amp;_nc_ss=7b2a8&amp;oh=00_AQMqFzK4UxMhT44RvA5O50by2GZEOppi7JT_fkYOZz_ENg&amp;oe=6ADBC31B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>61593860979577</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Frenchie forever</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61593860979577</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: frenchie, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>puppy (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>frenchie</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-11.fna.fbcdn.net/v/t39.30808-1/799279242_122105264901462032_3104521594671155506_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx543x551&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=OcnA7d5hAX4Q7kNvwEpUVDU&amp;_nc_oc=AdqY-GBfZGTKiHM5tZp_EHsD0kMZhxtg1I6WQBICs9vxVBVjmfVwipR7a8gIjnr5Gc0&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-11.fna&amp;_nc_gid=T8OyLSbfD_RUaywOpxI1wg&amp;_nc_ss=7b2a8&amp;oh=00_AQOYv3IaIX1X-3pz9E8yJXA8mE7WK0O0JJoN5i9GDINfDw&amp;oe=6ADBCA73</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>100083675791629</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Scherrer Sweet Doodles</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=100083675791629</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: doodles)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>doodles</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-10.fna.fbcdn.net/v/t39.30808-1/721779281_971577072308144_4733230633786410222_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1314x1313&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=zcWKcDg78YAQ7kNvwGF0LBH&amp;_nc_oc=Adqs7rDIFyoXBosBZzy4mDYARTzeCjxQhMY6pB4MGFYWajE-hVPeZQ4r0d3UybXlpNw&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-10.fna&amp;_nc_gid=T8OyLSbfD_RUaywOpxI1wg&amp;_nc_ss=7b2a8&amp;oh=00_AQNTKhxqJBj9H62Hr7qgsRgX4qi3GW_NMx8v9udi9i1CWA&amp;oe=6ADBBF7B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>61593966614797</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Heavenly Dachshunds</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/HeavenlyDachshunds</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: dachshunds)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>dachshunds</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-6.fna.fbcdn.net/v/t39.30808-1/801924750_122106295533465553_3582681563697098512_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1230x1230&amp;_nc_cat=102&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=KvJeIlfrCPYQ7kNvwGEgTvv&amp;_nc_oc=AdrVTz0ffQIZpDDTK_pbOXF_pd6mwd8tyvpvl_R2VwCCYEPXAJumF2wNAOnSgLEWQ4M&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-6.fna&amp;_nc_gid=T8OyLSbfD_RUaywOpxI1wg&amp;_nc_ss=7b2a8&amp;oh=00_AQPFT_HJ_DFw_MK6eBRI1qFag2Rp2DLDMqUWy5bWPiXc4A&amp;oe=6ADBDBCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>100092010588302</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Family Dog Vaycay Pet Sitting</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=100092010588302</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dog, P_dog=0.93)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>puppy (P=0.93)</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>0.9288</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>dog</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-6.fna.fbcdn.net/v/t39.30808-1/343973399_950772516342723_8863261499823246812_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx500x500&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=eSwhdLXll_sQ7kNvwEcxgcv&amp;_nc_oc=AdojpLfSaDkQcpq0dXtScMCVrG2CCD-cPjrPdBIMF7GQvF7_ViU_R31EDX4Lw2LkR2U&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-6.fna&amp;_nc_gid=wWKKYrquLNWzktadeOAp4g&amp;_nc_ss=7b2a8&amp;oh=00_AQNvx4rmp-ieAeelegpwil6D_E0Hf65Cf5sE2-a_SPxWCA&amp;oe=6ADBCE9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>61593185582221</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Ava the Australian Shepherd</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/avaaustralianshepherd</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: shepherd, australian shepherd, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>shepherd, australian shepherd</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-9.fna.fbcdn.net/v/t39.30808-1/819775887_122114813811439519_8141716067517529323_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx2047x2048&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=p8li4iTdwnEQ7kNvwGOgMWr&amp;_nc_oc=Adp2F8wdTjugRPzD0bNMOpnMfiTd3c1qxwrc2Z_im31ic63ngG4WAcUYTdhaxtV3tf8&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-9.fna&amp;_nc_gid=wWKKYrquLNWzktadeOAp4g&amp;_nc_ss=7b2a8&amp;oh=00_AQOHLlxgaBgXAGCehqQULypztjx-vCxcbA718UgF8PHhJQ&amp;oe=6ADBBDBB</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>100064337693424</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Karma's Dachshunds</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/KarmasDoxies</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dachshunds, dachshund, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>0.9999</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>dachshunds, dachshund</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-5.fna.fbcdn.net/v/t39.30808-1/464851534_940565858097995_8598999594224709224_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx2048x2048&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=ASrSVIkb3HEQ7kNvwFgnbI6&amp;_nc_oc=Adoch4h3Ftl9-TiJuXO22XIasOHjO7IVbInmD_Tn0c6Fa5k7H2fLAHlCQxC9ZUUPDoU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-5.fna&amp;_nc_gid=8FMi0KV6vUSSOBm5lOuUKg&amp;_nc_ss=7b2a8&amp;oh=00_AQMjqxsmLC5sIxVdXIEFRHFDEySzqhknfwQRVLS-aBJtIg&amp;oe=6ADBB327</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>61594091660932</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Gluten Off Lab doo</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61594091660932</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: lab)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>lab</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-11.fna.fbcdn.net/v/t39.30808-1/787542034_122203646186759747_6776481724409914524_n.jpg?stp=c31.0.1143.1143a_cp6_dst-jpg_tt6&amp;cstp=mx1143x1143&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=q-oEuSzTkuEQ7kNvwGJ6bad&amp;_nc_oc=Adr0wPHKwHVH2kapA2BuH_wCUg12PWgXYldRibPIM8_LWkdwxZ8l-jJ8Pbo7d8dk7Gg&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-11.fna&amp;_nc_gid=8FMi0KV6vUSSOBm5lOuUKg&amp;_nc_ss=7b2a8&amp;oh=00_AQPlMPTpBMCBO3OBTXP0ST6QJ7mD8rvLRrF_jbO18BdHcg&amp;oe=6ADBE3DE</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>61552188929671</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PNP Dachshunds LLC</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61552188929671</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dachshunds, P_dog=0.84)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>puppy (P=0.84)</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>0.8369</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>dachshunds</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-11.fna.fbcdn.net/v/t39.30808-1/485002964_122218989122072964_3967638820016736599_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx500x500&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=BdH9YpaNU3MQ7kNvwFBtMf0&amp;_nc_oc=Adq9e91hLjs3J3MQRBT41fhTXvoLhTPoRYc1Y2zXsstatMSXDuxXKnJW1GdhJFtIlME&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-11.fna&amp;_nc_gid=8FMi0KV6vUSSOBm5lOuUKg&amp;_nc_ss=7b2a8&amp;oh=00_AQOI78XEVRc7V6D4sflG_NssHJaD59PMTC8Ux8x1y1dczQ&amp;oe=6ADBD951</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>100077471214410</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Beaut Boxers</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/BeautBoxers</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: boxers)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>boxers</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-3.fna.fbcdn.net/v/t39.30808-1/819497572_1131867759405587_209993174050059485_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=lz59M37rZNEQ7kNvwGdbnNm&amp;_nc_oc=AdoYYENngNQu_4Gsjdy4WVB1aqV9cwuNZkSyBkssVX7Y6CnJy2mZsKamFEJMQhSdZgU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-3.fna&amp;_nc_gid=eWSb79gqwIoJ2uZMMRq1nw&amp;_nc_ss=7b2a8&amp;oh=00_AQMfWD_T72AY2YqyXbfDv9GRvW115vSIVC27mqFWQBZk3w&amp;oe=6ADBD021</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>61565119225294</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Magic Eagle Miniature Dachshunds</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/magiceagledoxies</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dachshunds, dachshund, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>dachshunds, dachshund</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-4.fna.fbcdn.net/v/t39.30808-1/783508002_122215974986503974_8899483936714065272_n.jpg?stp=c0.0.720.720a_cp0_dst-jpg_tt6&amp;cstp=mx720x720&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=ITID03AEcL0Q7kNvwGgRRxQ&amp;_nc_oc=AdoHqOw2CgyenWI6sdEcqlEk9x-3yCwcqXBJ2DW-TcLZ23kRBVu2ZhDPGyboOprdFzQ&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-4.fna&amp;_nc_gid=eWSb79gqwIoJ2uZMMRq1nw&amp;_nc_ss=7b2a8&amp;oh=00_AQOxUCyRwzN3CeXCoClV4Tq7bzKlHJdzSuv5TMrcnfNYAA&amp;oe=6ADBD6CF</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>61590471037312</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Loving Chihuahua Companions.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61590471037312</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: chihuahua, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>puppy (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>chihuahua</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-6.fna.fbcdn.net/v/t39.30808-1/843240300_122147696481349034_8275671350763553642_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx768x768&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Vu4xLttt6PgQ7kNvwFUC-We&amp;_nc_oc=AdqOxNLRckgXjza8ZcK0Lz96F-DfoSx1odmAWFvUXCnNIdRRWn9fOR0boZT0s9-XFxc&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-6.fna&amp;_nc_gid=eWSb79gqwIoJ2uZMMRq1nw&amp;_nc_ss=7b2a8&amp;oh=00_AQMwT4UoN24x1E0nxCfMrhc33zvw26HKucDKgFDkfmKzPA&amp;oe=6ADBBDBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>100067623948311</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Ivory &amp; Pine Goldens</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/IvoryandPineGoldens</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: goldens, golden retriever, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>goldens, golden retriever</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-7.fna.fbcdn.net/v/t39.30808-1/782615968_1384681697129282_5212663262034129488_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1933x1920&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=aZwKdecMfX8Q7kNvwG5E8rU&amp;_nc_oc=Adq7kNd4t1ND1PjvN0nHKyH2raeJ8L1sZnVWor_biV0RHIYu7RDoWHWMcr4tPGazhzA&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-7.fna&amp;_nc_gid=eWSb79gqwIoJ2uZMMRq1nw&amp;_nc_ss=7b2a8&amp;oh=00_AQOwthtfXNOmK8zSlpZtsV6ZgyjSv69YzY8-1kiPLrB9QQ&amp;oe=6ADBB77D</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>61591518293400</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>My Pawesome Boutique</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61591518293400</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Logo/Biển hiệu trại chó &amp; Từ khóa xác thực: dog, pet (không có mặt người)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.88)</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>dog, pet</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-5.fna.fbcdn.net/v/t39.30808-1/796969485_122127654063383943_1012761263205707610_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx2048x2048&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=cHm7XmwFU50Q7kNvwEoUe_2&amp;_nc_oc=AdqstLTGGiCAzkflZ3Pjw0stXtrU3TZgw2vJh6svpeM_2Mk9KD2Rv-QhCwEfPzbtkdA&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-5.fna&amp;_nc_gid=eWSb79gqwIoJ2uZMMRq1nw&amp;_nc_ss=7b2a8&amp;oh=00_AQOSCt9PCe2MHWNIqLHyyGoYUGwr-i7jaBWMX1YGK9dAEw&amp;oe=6ADBD8E7</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>61574790396010</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Gilded Glen Golden Retrievers</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61574790396010</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: golden retrievers, retrievers, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>puppy (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>golden retrievers, retrievers, goldens</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-11.fna.fbcdn.net/v/t39.30808-1/838966442_122181791750826346_2008532119779598613_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx2048x2043&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=jU4w85ESF-oQ7kNvwG2gvX1&amp;_nc_oc=Adr3sTnrhPSdyAzw-j-y3ExW8MG8eMOeGPZlTr-KbSagbRnXNBbMvUtcpUO9vS6c5aA&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-11.fna&amp;_nc_gid=rDRzbk4MF1d9kBrzrW4O6A&amp;_nc_ss=7b2a8&amp;oh=00_AQPTAhmdPbNl9Z2sr4IgdnAYJMvwQJik_mItbRyIh6puOQ&amp;oe=6ADBD19E</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>61591574075039</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Kristy's Cocker Spaniel</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61591574075039</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: cocker spaniel, cocker, P_dog=0.99)</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>puppy (P=0.99)</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>0.9916</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>cocker spaniel, cocker, spaniel</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-10.fna.fbcdn.net/v/t39.30808-1/738261667_122101295223385802_7358638121422389416_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=CIKSmJKyPIkQ7kNvwHcOv22&amp;_nc_oc=AdpPH7Y0j8iD3b6lwp4uiTLnRDYRZOC8FHr82Ni9ZMtluI9fiWtaGerIPaqXoEFShlQ&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-10.fna&amp;_nc_gid=rDRzbk4MF1d9kBrzrW4O6A&amp;_nc_ss=7b2a8&amp;oh=00_AQMTMU8sYl7DGxJuhWyJuuy4kiVbu17ZkilWJ5CVRug0Sg&amp;oe=6ADBE746</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>61593002885039</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Melissa's intelligence and loving golden retriever puppies for adoption</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61593002885039</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, golden retriever, retriever)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>puppy (P=0.98)</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>0.9846</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>puppies, golden retriever, retriever, puppy, dog, goldens</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-6.fna.fbcdn.net/v/t39.30808-1/775568628_122108102511433429_8072695245474966359_n.jpg?stp=c0.0.540.540a_cp0_dst-jpg_tt6&amp;cstp=mx540x540&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=xYTKzkWipWgQ7kNvwG8qTcY&amp;_nc_oc=AdrZz-GlnkMUONRpzLn-mdgcsWU74V3-vXTj4S6JObZrSbJybFr36H5jqaF65i1jipM&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-6.fna&amp;_nc_gid=rDRzbk4MF1d9kBrzrW4O6A&amp;_nc_ss=7b2a8&amp;oh=00_AQNVDuPqyIfVaa-VmsC1oc8Uv-MJo1ocySFjKGEScdk1cg&amp;oe=6ADBCE75</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>100057171741197</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>501 Shepherds</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/501shepherds</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: shepherds)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>shepherds</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-7.fna.fbcdn.net/v/t39.30808-1/724068393_1519028250012885_5132289179446813982_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1229x1229&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=TN9s3Sx1du0Q7kNvwHLKbKw&amp;_nc_oc=Adq-Mqq7owZSYO3LNDIQvn4U4kSRtApTHBHdPSWVvyrnWSkxaSaJ4j87bdXNjVVEMfI&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-7.fna&amp;_nc_gid=rDRzbk4MF1d9kBrzrW4O6A&amp;_nc_ss=7b2a8&amp;oh=00_AQM1-JB1suWJzyvHle3qfoyuGSu9pUIVLWWDrSs4le9HSQ&amp;oe=6ADBD364</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>100057622690855</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Doodle Denise Designs</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/doodledenisedesigns</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: doodle, P_dog=0.98)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>puppy (P=0.98)</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>0.9835</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>doodle</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-6.fna.fbcdn.net/v/t39.30808-1/771694472_1511430180787724_1527618184332262383_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx360x360&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=s39yCkZxl7AQ7kNvwG-_K0z&amp;_nc_oc=AdpzqqyE5utNWfKstVJejtxpFbB101y4p7RVpdlUlpocZmiwGseeAkXejwi5ElIMgh0&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-6.fna&amp;_nc_gid=rDRzbk4MF1d9kBrzrW4O6A&amp;_nc_ss=7b2a8&amp;oh=00_AQNKXAzIOKWXkQbgqY35fg_9V6oqnpIeIwLyerkJRhHDTg&amp;oe=6ADBB534</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>100082969255746</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sterling Run Retrievers</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SterlingRunRetrievers</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: retrievers)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>retrievers</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-6.fna.fbcdn.net/v/t39.30808-1/337398196_667116724869919_321658006795666061_n.jpg?stp=c40.40.770.770a_cp0_dst-jpg_tt6&amp;cstp=mx770x770&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=ofrjoYyYe5UQ7kNvwGppCOR&amp;_nc_oc=Adpqc310jk8Ul9RJdCphU-tSbIjWwTGP3NJZ5s_DbcRY-DSc5O5UT0iJVqq2MNGHbC8&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-6.fna&amp;_nc_gid=TDYxriTklat71Keid_AFYA&amp;_nc_ss=7b2a8&amp;oh=00_AQMKlu3KMTM7ROizGJhH2YrdvQSXpbLAEZDsY1MXZmPQOA&amp;oe=6ADBDEE4</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>100082062487155</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Kathryn,s Dachshunds</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=100082062487155</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: dachshunds)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>dachshunds</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-7.fna.fbcdn.net/v/t39.30808-1/792029861_1056334347111972_7582008765450913435_n.jpg?stp=c115.0.922.922a_cp0_dst-jpg_tt6&amp;cstp=mx922x922&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=L0Zi5NSWCoUQ7kNvwG3OJT_&amp;_nc_oc=AdpR7Yz6rLa2cEig3jmNww2ewh8uFc7pyBr9S60HWM2hzc21aYTcPQjSK0liDJuRQqU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-7.fna&amp;_nc_gid=TDYxriTklat71Keid_AFYA&amp;_nc_ss=7b2a8&amp;oh=00_AQNYYKOFVRw2jVXFtlzI-PpCCb6IK3UeTDHqaMumk0AU5Q&amp;oe=6ADBBD3B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>61590891808028</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Lil Debbies Darling Pets</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61590891808028</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>AI Thị giác nhận diện chó trưởng thành (Adult=0.98, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-7.fna.fbcdn.net/v/t39.30808-1/789034386_122120608101363060_6764403641595204862_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx765x768&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=XJdAslo7VmkQ7kNvwGA-4Jw&amp;_nc_oc=AdrPfm-GI35QztTTp_V9opzjQIGJRWlXqff6wIcCdCS9xwn1ODIaTkx7g9BieJmEcug&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-7.fna&amp;_nc_gid=TDYxriTklat71Keid_AFYA&amp;_nc_ss=7b2a8&amp;oh=00_AQNFUFp6AgEl0s_MfhL0AkuYKLrrx-QSKrZCNREMZyzFyA&amp;oe=6ADBD1C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>100063635496530</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>My Cavalier Puppies</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/CKCSpuppies</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, cavalier, puppy)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>puppy (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>puppies, cavalier, puppy, dog</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-6.fna.fbcdn.net/v/t39.30808-1/518654113_1292014406263064_7026757245242116044_n.jpg?stp=c183.0.733.733a_cp0_dst-jpg_tt6&amp;cstp=mx733x733&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=QMPH9tUW92sQ7kNvwEeb4LJ&amp;_nc_oc=AdofNmDHMz5p58sGMn8iGU9J0W9Z2Yfo7gq8hDIL6EtcyGbSWURPADWQA0QVHw_5U-Q&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-6.fna&amp;_nc_gid=DcywuF2wpVi51IbgKaoiHw&amp;_nc_ss=7b2a8&amp;oh=00_AQNKruxItNUgAEzN7zRgesffghgV4XANls_qRNmoci3HOQ&amp;oe=6ADBCBDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>61573687850343</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Lizzie’s Doxies</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/Lizziesdoxies</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: doxies, dachshund)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>doxies, dachshund</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn2-7.fna.fbcdn.net/v/t39.30808-1/722606315_122197262402789595_3440958979727817129_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=vo5jxlckh2AQ7kNvwHNTcBG&amp;_nc_oc=AdrxhFe0d-sRwKCtcxoJJagH1OSZ6v3fwnWY1aI2PkOOF3YaMuuSvHfd1zjpbJkJgEA&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn2-7.fna&amp;_nc_gid=DcywuF2wpVi51IbgKaoiHw&amp;_nc_ss=7b2a8&amp;oh=00_AQNV4w7oAkEVlLLzEaHbTGwCy42Hjsa4TYFE1oYeSUE5xw&amp;oe=6ADBE4AB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Decouple 3-tool architecture, build standalone Light-Mode Harvester UI with VI/ZH bilingual support, clean test videos
</commit_message>
<xml_diff>
--- a/data/verified_step1/step1_verified_dogs_latest.xlsx
+++ b/data/verified_step1/step1_verified_dogs_latest.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -438,7 +438,7 @@
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -495,40 +495,40 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>61594731538136</t>
+          <t>990587153326216</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cocker Spaniel</t>
+          <t>Stephanie’s Puppy Colony</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61594731538136</t>
+          <t>https://www.facebook.com/stephaniespuppycolony</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: cocker spaniel, cocker, P_dog=1.00)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppy, dog)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>adult_dog (P=1.00)</t>
+          <t>non_dog (P=0.95)</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>cocker spaniel, cocker, spaniel</t>
+          <t>puppy, dog</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/799676841_122095967409491051_5891965567465364453_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1290x1290&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Ymha57zXx_IQ7kNvwE75H-2&amp;_nc_oc=AdpGUknfutZcuNbtFir-EQiA4Fpb-CaowPGR2RXfWqhMsFwnXU_26gK-dI-wKQ7L1JQ&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=OzYFzMbeZJVf-lKCp-SPQw&amp;_nc_ss=7b2a8&amp;oh=00_AQNeWFbDXtU2-10Zz6hSG7j9u1IsICavyzOdmw1pyM6OfA&amp;oe=6ADD9673</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/696012345_990587153326216_235921294833267089_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=aikJ6ENAQrYQ7kNvwHzmK2b&amp;_nc_oc=AdqqI-iDUD_hCiFmrgfgCpz2hWtdR8rV0a0DxEPdwE1mZo-KRs6Ak6lHvuK-FE2l-bc&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQOhEGIqNeYTF1X7iMkn_MglHpgDQ_GKTEsAjekMf7PQYg&amp;oe=6ADE3155</t>
         </is>
       </c>
     </row>
@@ -538,40 +538,40 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>61595513098587</t>
+          <t>61595211969465</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>free dachshund puppies for adoption and rehoming</t>
+          <t>CaviCajun Kennels Cavapoos&amp;Cavaliers</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61595513098587</t>
+          <t>https://www.facebook.com/profile.php?id=61595211969465</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, dachshund, puppy)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: kennels, cavalier, poodle)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>puppy (P=1.00)</t>
+          <t>puppy (P=0.95)</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.9993</v>
+        <v>0.95</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>puppies, dachshund, puppy, dog</t>
+          <t>kennels, cavalier, poodle, cavapoo</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/853444971_122096623407517103_2508650680056135816_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx2026x2048&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=mQc1kpvezdMQ7kNvwHZRa0X&amp;_nc_oc=Adpo3LNNAhd_KH1qGnc7tEnHME9Zsucl2edBgrcaDgrMrOZycKl1ru__TaGElpvYdmI&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=OzYFzMbeZJVf-lKCp-SPQw&amp;_nc_ss=7b2a8&amp;oh=00_AQP_mRDcdtHIIcJy0PAqbPrV-xEYPoP0ZZu3lo742mSUWA&amp;oe=6ADD93C7</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/848993890_122103405711507065_2101132370405643345_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1094x1104&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=wmrDpQCvqlQQ7kNvwFOxhqS&amp;_nc_oc=Adrla7AbjZzoN3_2yJ034He_jcO1yaI3lkyAOaetgAU7c9X3M3kav7YZAhHw8_lZr5M&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQOEqW7QtF7l9HwdoYHNGGLzuQxBC5czwDBO2clPwQ2ZLw&amp;oe=6ADE4358</t>
         </is>
       </c>
     </row>
@@ -581,40 +581,40 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>100082804552805</t>
+          <t>1042413175162171</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Chandra K9 Commando Working Dog Kennel Bengaluru</t>
+          <t>Redhill Boykin Spaniels</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=100082804552805</t>
+          <t>https://www.facebook.com/RedhillBoykinSpaniels</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>B2B Breeder / Trại chó xác thực qua NLP &amp; Từ khóa (dog, k9, kennel)</t>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: boykin, spaniels)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>puppy (P=1.00)</t>
+          <t>non_dog (P=0.85)</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>dog, k9, kennel, working dog</t>
+          <t>boykin, spaniels</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/440336552_418005740969574_7966871653006742989_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=TSqss9UjjzMQ7kNvwEqAW_7&amp;_nc_oc=Adp1iZ3SualCnXsqbDmCfPhvxWtXtDKpSCOGgLhSZNY1MTbEDNoIkIoUZgfIASzZ3vg&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=OzYFzMbeZJVf-lKCp-SPQw&amp;_nc_ss=7b2a8&amp;oh=00_AQPajJCoARtRJJ9fnm47pW2DKfmZnaypS230qW_9fjm2Og&amp;oe=6ADD9901</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/780104405_1042413175162171_4016551396372726401_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Hgx53HAhos4Q7kNvwG7ULQ1&amp;_nc_oc=AdpiS4cY3jkx_YKrdp-Rj9a1puGI7YMNbmqeVw3eUC5EWiDLsTL54FCIBp6YfR7Be5Y&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQOQxEkwjDSowV8otco6c1JQ56-v5vGWyYuek0bVXHOn6g&amp;oe=6ADE4DFE</t>
         </is>
       </c>
     </row>
@@ -624,40 +624,40 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>61595221846060</t>
+          <t>61552753361052</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Greenhouse Yorkies</t>
+          <t>Eliana’s Shih Tzu Home</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61595221846060</t>
+          <t>https://www.facebook.com/profile.php?id=61552753361052</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: yorkies, P_dog=0.57)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: shih tzu, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>adult_dog (P=0.57)</t>
+          <t>adult_dog (P=1.00)</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.5735</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>yorkies</t>
+          <t>shih tzu</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/853675465_122107209423507394_8773063100519475064_n.jpg?stp=c0.0.736.736a_cp0_dst-jpg_tt6&amp;cstp=mx736x736&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=bB8XyIMvgRsQ7kNvwGim8JX&amp;_nc_oc=AdoTjxZ2WxtuRe32c29II2VguQWs76Y2BUjM_tvPdgg7yAGJ5sOwFJhduCcJmR7a19E&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=fhmXFF3Ink9ZXE2wPEBPpQ&amp;_nc_ss=7b2a8&amp;oh=00_AQNsEn5_nWdrZUc4VnYs6PKbrCUmlExBTWSNOvwf2ngLJA&amp;oe=6ADDB286</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/838967521_122256247310091778_3876985609640057852_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1320x1320&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=1zSXN-tHW60Q7kNvwH-KUnB&amp;_nc_oc=Adrc_fhEGh1mGV1c3FFbYPc5uIAxmk8GO6m7mBgQ7fdJH3Ty_8f1QYh3GZO-pNFxepM&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQOZcfg42vUA05lqNSqu4Y70ZV55QgWmYsRDhYrkhjoCjw&amp;oe=6ADE65A5</t>
         </is>
       </c>
     </row>
@@ -667,40 +667,40 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>61595352087577</t>
+          <t>909141020535285</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>𝐑𝐑𝐨𝐬𝐞𝐰𝐨𝐨𝐝 𝐅𝐚𝐦𝐢𝐥𝐲 𝐏𝐨𝐨𝐝𝐥𝐞𝐬</t>
+          <t>Family Loved Golden Retrievers</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61595352087577</t>
+          <t>https://www.facebook.com/FamilyLovedGoldenRetrievers</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: poodles)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: golden retrievers, retrievers, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>non_dog (P=0.85)</t>
+          <t>adult_dog (P=1.00)</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>poodles</t>
+          <t>golden retrievers, retrievers, goldens</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/841343199_122096667393511736_1512305433899181321_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1024x1024&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=he-uNEKilPwQ7kNvwE9YVQQ&amp;_nc_oc=AdrUG9Gu0qAD4bm9caItGxTLIR7AMgGTpbK7KcS1TbCj-OuoZTbiKSyJXpewD5wqAvc&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=qX2cURIoXveZ8q3ypB7H8g&amp;_nc_ss=7b2a8&amp;oh=00_AQMvvm2AE9kQ2p2xrwI0TP-vSOT6TE4BI-3eYD0GIIlkLA&amp;oe=6ADD853E</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/326488783_909141020535285_7958935178343501974_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=KCkBpAyH_X4Q7kNvwG_0u7p&amp;_nc_oc=AdqpaFrDKUJWZ0RjZaw1Ftlhn-WNPFO_xA6h11WNnO0orGxBODdWYLepdmmoMZCNvhU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQMIEW37_fVuRYohQzq54OCkEnN8kOT6qgITq91MNuE5tg&amp;oe=6ADE55C8</t>
         </is>
       </c>
     </row>
@@ -710,31 +710,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>61594231833777</t>
+          <t>61591593760286</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Soft For Dogs</t>
+          <t>I Love Dogs Forge 'N Fetch</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61594231833777</t>
+          <t>https://www.facebook.com/profile.php?id=61591593760286</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Logo/Biển hiệu trại chó &amp; Từ khóa xác thực: dogs (không có mặt người)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dogs, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>non_dog (P=0.88)</t>
+          <t>puppy (P=1.00)</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0.88</v>
+        <v>1</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/802072198_122099903445474394_6740119027340512439_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1080x1080&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=rcCG6sSZoRIQ7kNvwGM6gQC&amp;_nc_oc=AdqR-BTMwbz-9Aiz9ezsZ8NJrBHKMNmpV-HfjJj39gaqnj8aN6hYBIAfP72LD3tAZ-k&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=5YXrbTSB9IDYBoSM_3Pp2Q&amp;_nc_ss=7b2a8&amp;oh=00_AQMRwWS84imM2_pXxgdzwhIK3ZaJkA4Qb6-mEBYeh6Eiqg&amp;oe=6ADD8C21</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/753954046_122112615273386458_4146374115223244916_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1079x1078&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Ni6iO7UEIhAQ7kNvwEX3aDq&amp;_nc_oc=Adrz8cAAO2KmFnkZuRFza8iqAvdl16K9ANiruVQlW0Gf0J8H84W8375VrlBdRXWu9Uo&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=HP3imHJzQbwK5_D9L5y4YQ&amp;_nc_ss=7b2a8&amp;oh=00_AQO2tZAE_PYlpJU34MDZlFQD15hI23WOU7elgwST5qh6bw&amp;oe=6ADE430D</t>
         </is>
       </c>
     </row>
@@ -753,40 +753,40 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>61595290116794</t>
+          <t>61594775080228</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dachshund Puppies</t>
+          <t>Yorkshih Pupco</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61595290116794</t>
+          <t>https://www.facebook.com/profile.php?id=61594775080228</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, dachshund, puppy)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: breeder, breeders, pupco)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>adult_dog (P=1.00)</t>
+          <t>non_dog (P=0.95)</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>puppies, dachshund, puppy, dog</t>
+          <t>breeder, breeders, pupco, yorkshire, shih tzu, pup, puppy, dog</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/853053396_122102754147509670_4567344291178019063_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1440x1440&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=W5qnkOd7qBsQ7kNvwFN9Goh&amp;_nc_oc=Adp5jXl5s2yJ4q7I28E2_oTqjqm-XINrrawXKX8qltpS6k4S8wCKSA3pvYBHqKTAKi0&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=5YXrbTSB9IDYBoSM_3Pp2Q&amp;_nc_ss=7b2a8&amp;oh=00_AQPpBwkHSIwD5t77bIJBr7GNNOXT9pTfLZ5Cs1doB5AHHg&amp;oe=6ADDAA7C</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/830513831_122102418099492502_4902222354387580447_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx800x800&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=EsJnYIDH-P0Q7kNvwF_S4j8&amp;_nc_oc=AdolxT1vtUo6WEzYifsxx3wdxMH5qMFOkvd3Dv6_4e8LN-DXvU8v0UGTTe9ILvMYdig&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=HP3imHJzQbwK5_D9L5y4YQ&amp;_nc_ss=7b2a8&amp;oh=00_AQMxPuNOASl5lLsgUP07MQPcBGYSzfk1IVucqOeJFMC7Vw&amp;oe=6ADE47B5</t>
         </is>
       </c>
     </row>
@@ -796,40 +796,40 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>61595289693197</t>
+          <t>61551532070511</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Paradise Frenchies</t>
+          <t>Oakhaven Acres Aussies- AKC Australian Shepherds</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61595289693197</t>
+          <t>https://www.facebook.com/profile.php?id=61551532070511</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: frenchies, frenchie)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: akc, shepherds, aussies)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>non_dog (P=0.85)</t>
+          <t>non_dog (P=0.95)</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.85</v>
+        <v>0.95</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>frenchies, frenchie, french bulldog</t>
+          <t>akc, shepherds, aussies, australian shepherd</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/848995038_122099228025509656_4048205347987609657_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx640x640&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Fv4WV33GQWgQ7kNvwEv4qzX&amp;_nc_oc=AdrYYYPMyjK3d_DgwPY9BXatJnkie0jHpuHTJ9pvm75P0dPzVpOJmpn_DES7ZUwB7BM&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=5YXrbTSB9IDYBoSM_3Pp2Q&amp;_nc_ss=7b2a8&amp;oh=00_AQNl8V2nFNTA-b9B-pkwF8pBbhDwHZgyNUWAp3-ML6Cy6Q&amp;oe=6ADDA41C</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/427143042_122133778058051069_7335697382670797595_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1170x1170&amp;_nc_cat=102&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=FXFGb8mH_kEQ7kNvwGyHi8Y&amp;_nc_oc=Adr7QPqn9TWmoPvg5PVMQ0XhE5o0u6TghXQJDLA6BUNVWjNBCwYGYaq3OEn_ED4uQBQ&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=HP3imHJzQbwK5_D9L5y4YQ&amp;_nc_ss=7b2a8&amp;oh=00_AQPI-hF_GlM-ASJS-S_YyieWtSZ-BN8gDQKxOwDEdZiD9Q&amp;oe=6ADE3592</t>
         </is>
       </c>
     </row>
@@ -839,40 +839,40 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>61594332256058</t>
+          <t>61588242310496</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>German Shepherd World</t>
+          <t>Bottom Top Basset’s</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61594332256058</t>
+          <t>https://www.facebook.com/profile.php?id=61588242310496</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: german shepherd, shepherd, P_dog=0.89)</t>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: basset)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>puppy (P=0.89)</t>
+          <t>non_dog (P=0.85)</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.8907</v>
+        <v>0.85</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>german shepherd, shepherd</t>
+          <t>basset</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/845925005_122118219585477741_7967768453723125043_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=HflOslV30asQ7kNvwFtZQYz&amp;_nc_oc=AdreAgC6WxrN9g0mmdn_4edELu3837jsqawtp-noYL_XuakaVzqSac3qjlEwf2YMTl8&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=5YXrbTSB9IDYBoSM_3Pp2Q&amp;_nc_ss=7b2a8&amp;oh=00_AQPEwHkwOF4qCxKv9-vrv6IWX41c_vSEXj86mmoEg2NiIw&amp;oe=6ADD876C</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/825267903_122124942699274743_5172081817443253017_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=2Nx0sQfNEdYQ7kNvwEEHpwQ&amp;_nc_oc=AdrGG7ydqjr2dqoG-wqqKcuIg7HL53ZRvs1rZ-bH9HiCb8i1oCMaFNiwOeeYbo3oF-8&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=d0EBryXU1UgygpoH5zQ81A&amp;_nc_ss=7b2a8&amp;oh=00_AQMClSH_3Pr7Fo8AETARMoZoeLNCTt3jcoMjIHQnaOycgg&amp;oe=6ADE5311</t>
         </is>
       </c>
     </row>
@@ -882,22 +882,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>100076508311524</t>
+          <t>61594781858150</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Golden Acres Poodle Farm</t>
+          <t>Pawsome Daschund Puppies</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=100076508311524</t>
+          <t>https://www.facebook.com/profile.php?id=61594781858150</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: poodle, goldens, P_dog=1.00)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, puppy, dog)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -910,12 +910,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>poodle, goldens</t>
+          <t>puppies, puppy, dog</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/467616410_586656400561299_7608861023452401031_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1536x1536&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=DyEWKZ-Grj4Q7kNvwFm_K9C&amp;_nc_oc=Adqq3Tum4IVuxbmj4xYpZ9WpR1BfyFXu6hX_wpSoZ8Wf2OACCK9Jz2fs4E10oe9mRXU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=c87bpxjG87PHL7f6oGAZnA&amp;_nc_ss=7b2a8&amp;oh=00_AQNyibrJCO1a34DlH-LpivM-brzQM7GIP7rlSlT34IJRsQ&amp;oe=6ADD856B</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/839806917_122108759649492728_2289165301397021762_n.jpg?stp=c0.0.540.540a_cp0_dst-jpg_tt6&amp;cstp=mx540x540&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=2UvAoPM99EEQ7kNvwHxkrkL&amp;_nc_oc=AdrESu6ut2JVf7qtFuvRkFUswJlaQsHriYHFk6b4MTqBZbGWen-GSMMdPRKni2uuexU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=y4c-DeRUU11dMr2UX5j8JA&amp;_nc_ss=7b2a8&amp;oh=00_AQOcoHhyZy0YKhN_sW7QUn2AkPK_Kt9grNoXmvOIjVca6w&amp;oe=6ADE3700</t>
         </is>
       </c>
     </row>
@@ -925,22 +925,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>61594975678956</t>
+          <t>61594195772352</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ABC VIP DOGS</t>
+          <t>Jose MiniPuppies</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61594975678956</t>
+          <t>https://www.facebook.com/profile.php?id=61594195772352</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dogs, P_dog=1.00)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppy, dog)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -949,16 +949,16 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>0.9996</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>dogs</t>
+          <t>puppy, dog</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/855164329_122110907037499189_877532196647671267_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1145x1146&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=5eKwegKjQesQ7kNvwG6OmjZ&amp;_nc_oc=Adr791HwdvEcX3kI8Uakb6zOhBK1g_1GzYmngDfNdOuYLEX4GzXMV5MEje7f_h4e7PY&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=c87bpxjG87PHL7f6oGAZnA&amp;_nc_ss=7b2a8&amp;oh=00_AQO2M9yk1JYAS2Er27WrImuYK0P3rAa393X0C7pvxST2ig&amp;oe=6ADDAB34</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/855646238_122124401871473192_6657591073014986332_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1053x1050&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=fpciUtL0RqgQ7kNvwHvDvml&amp;_nc_oc=AdrkOtpO68tVOeHRBbQwGKPXDMKv6JIvACChqv-71ZDlzMeiB7o2zM5DLwzGe9EmfD0&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=y4c-DeRUU11dMr2UX5j8JA&amp;_nc_ss=7b2a8&amp;oh=00_AQMoTuCS5W_fKqhvV4ISSWCagCN3T9NI57HCSPDhZ-PTug&amp;oe=6ADE44CF</t>
         </is>
       </c>
     </row>
@@ -968,40 +968,40 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>61595707163197</t>
+          <t>1489668089832323</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Lakeland Terrier México “Apolo’s Kennel”</t>
+          <t>Tambali Pembroke welsh corgis est. 1998</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61595707163197</t>
+          <t>https://www.facebook.com/Tambalicorgis</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: kennel, terrier)</t>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: corgis, pembroke)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>puppy (P=1.00)</t>
+          <t>non_dog (P=0.85)</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>kennel, terrier</t>
+          <t>corgis, pembroke</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/856470882_1773914520573760_7422947113457391568_n.jpg?stp=c102.0.819.819a_cp0_dst-jpg_tt6&amp;cstp=mx819x819&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=FshYNu6WXGYQ7kNvwEr-ckj&amp;_nc_oc=AdqkcB7O6QYjx1skN5BVUUh2-E725fSZ8XPu_aCQfwfEtf5wm6B2d_GkVicPXatP6zU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=FXpsU-C4WHklfFJi9gwJnA&amp;_nc_ss=7b2a8&amp;oh=00_AQMj1o6d6gKHb4XGveQ93Kpjk_cgONZVeQ6yF0_0VjMhmw&amp;oe=6ADDAFD8</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/628787013_1489668089832323_6013872381075739493_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1024x1024&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=78QAEnU19pYQ7kNvwEdF6M8&amp;_nc_oc=AdqAnBQs8chVNgaUNDOr8kq6u2kY2oQbBOhBaUC2ubsjg00tY22Uoqr4BrypC7ogkqs&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=y4c-DeRUU11dMr2UX5j8JA&amp;_nc_ss=7b2a8&amp;oh=00_AQOjodBjmS0_j0jf04e6FFQTcRlWSJdebAz-hS_2oJMDmQ&amp;oe=6ADE43E7</t>
         </is>
       </c>
     </row>
@@ -1011,40 +1011,40 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>61594915838249</t>
+          <t>61591427093472</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Lone Wolf Breeders</t>
+          <t>Franklineschipperkes Kennel</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61594915838249</t>
+          <t>https://www.facebook.com/profile.php?id=61591427093472</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: breeders)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: kennel)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>non_dog (P=0.95)</t>
+          <t>adult_dog (P=1.00)</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>breeders</t>
+          <t>kennel</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/834526337_4533280666990767_3514549822735751705_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx2000x2000&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=e5HOzZ7aqDYQ7kNvwFuIwkZ&amp;_nc_oc=AdrVKGHkEW0WKmTMXZR4TsSU1iwRmKg4Y5iQ8ixGaLqTtelyN_NfKPk1Ss9MQ3O6-gM&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=lUlIPiuATfIiJ4DmKfT7jg&amp;_nc_ss=7b2a8&amp;oh=00_AQPKpaExbgEjnMFR0E0Th96WvxMPTCc34l7L7lrxgFJm4w&amp;oe=6ADDA91F</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/818936768_122125355133380903_6137241591030814058_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx845x845&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=hekGuXarAzkQ7kNvwHSLKZB&amp;_nc_oc=AdqK_Pk1Vju7cJ78k38AbjiQxUPrgFfqzKFFtHS2yrhswAlzj4zAGl4mSWwr17GgtnE&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=y4c-DeRUU11dMr2UX5j8JA&amp;_nc_ss=7b2a8&amp;oh=00_AQMzIJk4OUXN4yGcWHszoK85mTqgYKndymGkEqsoTNLJQA&amp;oe=6ADE4719</t>
         </is>
       </c>
     </row>
@@ -1054,22 +1054,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>122093871489524357</t>
+          <t>61593315111061</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dolly Baby K9</t>
+          <t>Dachshund Puppies For Adoption And Rehoming</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/dollybaby.k9</t>
+          <t>https://www.facebook.com/profile.php?id=61593315111061</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: k9, P_dog=1.00)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, dachshund, puppy)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1082,12 +1082,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>k9</t>
+          <t>puppies, dachshund, puppy, dog</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/853578531_122093871489524357_34586254437558028_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx2045x2045&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=-7CGtPEIG2oQ7kNvwGfqgj7&amp;_nc_oc=Adp0CBstvJhKh3O4TgAx-nAE5qicnpjYjbP1gnMVo8B_tHfpYeL5n5cx13xlqwI_fzw&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=TgUWhg1SebUjfM7T33oocg&amp;_nc_ss=7b2a8&amp;oh=00_AQOxh-NOuP7ZUZ8fFeBmaWXQnMkDEL4J05LDJ58OrhKyKw&amp;oe=6ADD9FD0</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/766890471_122093395911443837_496170756872224230_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx828x828&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=ihYNssPKU28Q7kNvwEDZvlm&amp;_nc_oc=AdqfWpLpHPGHmq5J1VKT75IRA-swUUjpIjvWsYT90OxxjutYdMMbhfsCNAn4PNy0MWw&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=te8O4haIQ4bk8DSKcpSW7w&amp;_nc_ss=7b2a8&amp;oh=00_AQPNEnh89ueLb2hAllV42UGJvYLcE2NzbTXbGNnpUNbBcg&amp;oe=6ADE644E</t>
         </is>
       </c>
     </row>
@@ -1097,22 +1097,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>61590419896312</t>
+          <t>61594494459425</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Elite schnauzers rescue and rehoming</t>
+          <t>Autumn's Aussies</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61590419896312</t>
+          <t>https://www.facebook.com/profile.php?id=61594494459425</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: schnauzers, P_dog=1.00)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: aussies, australian shepherd, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1125,12 +1125,12 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>schnauzers</t>
+          <t>aussies, australian shepherd</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/724194389_122110156515347329_8649130341916381884_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1122x1123&amp;_nc_cat=102&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=xW_6qi_H5e4Q7kNvwEssLh2&amp;_nc_oc=AdpA_9mf_FS6lPe0OAd1y1tgdYQ0FI7UJN46Tw8OdA8xQrTExJ5WLAJ2IKORHhsE6bI&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=8AMkU5dntGptVHluBOghoA&amp;_nc_ss=7b2a8&amp;oh=00_AQMhuDm_n4qQ_jAHavwe08OA9H02h91HaVZtfvK5NsAGRA&amp;oe=6ADDA89B</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/820934527_2313498826091469_1498160885209143484_n.jpg?stp=c0.0.1536.1536a_cp0_dst-jpg_tt6&amp;cstp=mx1536x1536&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=L03VojkGVZUQ7kNvwEmEWpp&amp;_nc_oc=AdpipHwllV-m4oMIMNa0_C0eG8SYzQy-oJfiT01OuEgrzjRX2jTN7jORBhtWizMu61Y&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=te8O4haIQ4bk8DSKcpSW7w&amp;_nc_ss=7b2a8&amp;oh=00_AQNfQcVVHLnK9yS2OtyTyFQgwP57d7A1ktjz9h38oZnzCQ&amp;oe=6ADE3FE9</t>
         </is>
       </c>
     </row>
@@ -1140,40 +1140,83 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>61595452472675</t>
+          <t>122193681896610895</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pirate Paws Grooming</t>
+          <t>Knock &amp; Bark Miniature Schnauzer.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61595452472675</t>
+          <t>https://www.facebook.com/knockandbark</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: grooming, P_dog=0.99)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: schnauzer, miniature schnauzer, P_dog=0.97)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>puppy (P=0.99)</t>
+          <t>puppy (P=0.97)</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0.9918</v>
+        <v>0.9741</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>grooming</t>
+          <t>schnauzer, miniature schnauzer</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn9-1.fna.fbcdn.net/v/t39.30808-1/853048787_122099219925515082_8756659190000181024_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1122x1122&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=0jh7DvbrDsYQ7kNvwE4lQyX&amp;_nc_oc=Ado7fFc3THZO5EG5QEeKo_IEwWlYhzmJHvU8I6vW45Hb8k_1UC8WOaiAON-RH7rJFmM&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn9-1.fna&amp;_nc_gid=8AMkU5dntGptVHluBOghoA&amp;_nc_ss=7b2a8&amp;oh=00_AQNGtrPFr_KwF_pccehe1nDymlRpDGwXrlRfeAMbj4Ib8A&amp;oe=6ADD928D</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/779082815_122193681896610895_1254854747032187011_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1134x1122&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=N6pIjA1Ts40Q7kNvwGdzE7P&amp;_nc_oc=AdrKeMKHlIsY0Br3XkfOG2hxdtvMcmsaoRr84NZDJtCAPggWhjKVPK2mvbARdKt8b_A&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=te8O4haIQ4bk8DSKcpSW7w&amp;_nc_ss=7b2a8&amp;oh=00_AQOOfR66vg0y_jnCql9iGHPoPUknemKeAXcUGQCJ5PiMOw&amp;oe=6ADE2F3C</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>61593913773814</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Responsible Breeder Mentorship Program</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=61593913773814</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: breeder)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.95)</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>breeder</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/789960755_10215640356039617_8106197547239706512_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Ch42QEEATugQ7kNvwFkzIiS&amp;_nc_oc=Adphq4c8PLfRYPgEWIBtAJ-M8vh4V2BGW3LeogcZpQlX8eo9WjUJSbS0GNyPedmjw2I&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=te8O4haIQ4bk8DSKcpSW7w&amp;_nc_ss=7b2a8&amp;oh=00_AQN5vX4_YYWjLBxPJO8dxEdp3cxECEz9Rb-Q5FKwVbRF9w&amp;oe=6ADE3182</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: sync robust facebook url normalization and active:false side-tab realtime streaming
</commit_message>
<xml_diff>
--- a/data/verified_step1/step1_verified_dogs_latest.xlsx
+++ b/data/verified_step1/step1_verified_dogs_latest.xlsx
@@ -428,17 +428,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="41" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -495,40 +495,40 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>990587153326216</t>
+          <t>1596373112283090</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Stephanie’s Puppy Colony</t>
+          <t>Firestorm Goldens</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/stephaniespuppycolony</t>
+          <t>https://www.facebook.com/Firestormgoldenretrievers</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppy, dog)</t>
+          <t>Logo/Biển hiệu trại chó &amp; Từ khóa xác thực: goldens, golden retriever (không có mặt người)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>non_dog (P=0.95)</t>
+          <t>non_dog (P=0.88)</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>0.95</v>
+        <v>0.88</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>puppy, dog</t>
+          <t>goldens, golden retriever</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/696012345_990587153326216_235921294833267089_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=aikJ6ENAQrYQ7kNvwHzmK2b&amp;_nc_oc=AdqqI-iDUD_hCiFmrgfgCpz2hWtdR8rV0a0DxEPdwE1mZo-KRs6Ak6lHvuK-FE2l-bc&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQOhEGIqNeYTF1X7iMkn_MglHpgDQ_GKTEsAjekMf7PQYg&amp;oe=6ADE3155</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/760620948_1596373112283090_8124428097826053721_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx2048x2048&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=vQnoXfeIIAsQ7kNvwHIoe36&amp;_nc_oc=AdrRtHloFKO14oKmFm4hrxLJpVJ4J7kh_TzW0hNMYCZans0AfawhWRHo7Z3aypBJT94&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=wvBxwXYC6uM7D2fsdOPfcA&amp;_nc_ss=7b2a8&amp;oh=00_AQOkNojq6ZxWDllkdngCdZ4PW99tEfnO33OsWHCSOcAGlQ&amp;oe=6ADE3BAE</t>
         </is>
       </c>
     </row>
@@ -538,40 +538,40 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>61595211969465</t>
+          <t>1058086863465242</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CaviCajun Kennels Cavapoos&amp;Cavaliers</t>
+          <t>Smooches for Pooches</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61595211969465</t>
+          <t>https://www.facebook.com/loveofpups</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: kennels, cavalier, poodle)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppy, dog, puppies)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>puppy (P=0.95)</t>
+          <t>adult_dog (P=1.00)</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>kennels, cavalier, poodle, cavapoo</t>
+          <t>puppy, dog, puppies</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/848993890_122103405711507065_2101132370405643345_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1094x1104&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=wmrDpQCvqlQQ7kNvwFOxhqS&amp;_nc_oc=Adrla7AbjZzoN3_2yJ034He_jcO1yaI3lkyAOaetgAU7c9X3M3kav7YZAhHw8_lZr5M&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQOEqW7QtF7l9HwdoYHNGGLzuQxBC5czwDBO2clPwQ2ZLw&amp;oe=6ADE4358</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/773486111_1058086863465242_344051957738859922_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1086x1086&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Q7quceSoaj4Q7kNvwF9pNK7&amp;_nc_oc=Adowdu5feQlQuIM8cMskP7WX5FjSWMgEsv_sozqn4lbdoomeyZZ9i1cgkZALzQ_EcJw&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=wvBxwXYC6uM7D2fsdOPfcA&amp;_nc_ss=7b2a8&amp;oh=00_AQPT5aTSyALYre6DBDFzRfYcLpomB41eaR0Yd_XXP1HpHg&amp;oe=6ADE5BEE</t>
         </is>
       </c>
     </row>
@@ -581,40 +581,40 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1042413175162171</t>
+          <t>122095855856933094</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Redhill Boykin Spaniels</t>
+          <t>Bailey’s Cajun Canines LLC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/RedhillBoykinSpaniels</t>
+          <t>https://www.facebook.com/Baileyscajuncaninesllc</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: boykin, spaniels)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: canines, P_dog=0.97)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>non_dog (P=0.85)</t>
+          <t>puppy (P=0.97)</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>0.85</v>
+        <v>0.972</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>boykin, spaniels</t>
+          <t>canines</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/780104405_1042413175162171_4016551396372726401_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Hgx53HAhos4Q7kNvwG7ULQ1&amp;_nc_oc=AdpiS4cY3jkx_YKrdp-Rj9a1puGI7YMNbmqeVw3eUC5EWiDLsTL54FCIBp6YfR7Be5Y&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQOQxEkwjDSowV8otco6c1JQ56-v5vGWyYuek0bVXHOn6g&amp;oe=6ADE4DFE</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/514361430_122095855856933094_4776262354102086972_n.jpg?stp=c28.0.1160.1160a_cp0_dst-jpg_tt6&amp;cstp=mx1160x1160&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=m0gI9fOCmkoQ7kNvwGO-eGL&amp;_nc_oc=AdqJQi32T0aUKVaL0X8svdciqgtz6-VRtlNQtRrFAGJkrxaU99PDIDKzTD8ht5sJWus&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=pelMvMZbxRbN5uMQAHbS1Q&amp;_nc_ss=7b2a8&amp;oh=00_AQPUrI0rX38UHxgde2mbt26ygN76wHf49g8rVFWk6NIEZw&amp;oe=6ADE463A</t>
         </is>
       </c>
     </row>
@@ -624,40 +624,40 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>61552753361052</t>
+          <t>1117686188781662</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eliana’s Shih Tzu Home</t>
+          <t>Doodles of Louisiana</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61552753361052</t>
+          <t>https://www.facebook.com/DoodlesOfLouisiana</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: shih tzu, P_dog=1.00)</t>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: doodles)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>adult_dog (P=1.00)</t>
+          <t>non_dog (P=0.85)</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>shih tzu</t>
+          <t>doodles</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/838967521_122256247310091778_3876985609640057852_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx1320x1320&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=1zSXN-tHW60Q7kNvwH-KUnB&amp;_nc_oc=Adrc_fhEGh1mGV1c3FFbYPc5uIAxmk8GO6m7mBgQ7fdJH3Ty_8f1QYh3GZO-pNFxepM&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQOZcfg42vUA05lqNSqu4Y70ZV55QgWmYsRDhYrkhjoCjw&amp;oe=6ADE65A5</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/280485787_1117686188781662_1773497406171536734_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx958x958&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=LvizzZ2jb68Q7kNvwG_-9za&amp;_nc_oc=AdrZ-6_n-rmjW0KFAoW248Qa7-Eczl9XNgE3CdB6Cq7AoXc4Fs6vhLSe-W2mKmgREGY&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=pelMvMZbxRbN5uMQAHbS1Q&amp;_nc_ss=7b2a8&amp;oh=00_AQM9fvnyUQYVOsjpJy_ToFyAqhYK3KsK0rzWs8DVS57_BQ&amp;oe=6ADE69C2</t>
         </is>
       </c>
     </row>
@@ -667,22 +667,22 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>909141020535285</t>
+          <t>122348323874064888</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Family Loved Golden Retrievers</t>
+          <t>16 Paws Goldens</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/FamilyLovedGoldenRetrievers</t>
+          <t>https://www.facebook.com/16PawsGoldens</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: golden retrievers, retrievers, P_dog=1.00)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: goldens, golden retriever, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -695,12 +695,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>golden retrievers, retrievers, goldens</t>
+          <t>goldens, golden retriever</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/326488783_909141020535285_7958935178343501974_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=KCkBpAyH_X4Q7kNvwG_0u7p&amp;_nc_oc=AdqpaFrDKUJWZ0RjZaw1Ftlhn-WNPFO_xA6h11WNnO0orGxBODdWYLepdmmoMZCNvhU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=TwICOsyVNFPr1QMO3-Kemw&amp;_nc_ss=7b2a8&amp;oh=00_AQMIEW37_fVuRYohQzq54OCkEnN8kOT6qgITq91MNuE5tg&amp;oe=6ADE55C8</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/853441685_122348323874064888_3226424898471433872_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx2048x2048&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=12YKDZ0y3MoQ7kNvwE4F8SH&amp;_nc_oc=AdrfUphicb9s0yPRDTKRQnAvg71twQHzKlsle2Vw5awfEH_wJTAAcLXSKsN9Sw-esN0&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=pelMvMZbxRbN5uMQAHbS1Q&amp;_nc_ss=7b2a8&amp;oh=00_AQPwNvT5R7xJXZlNuaZ4yyZlfF4OD0i7s4Y4_3A1PRpPOQ&amp;oe=6ADE3E17</t>
         </is>
       </c>
     </row>
@@ -710,40 +710,40 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>61591593760286</t>
+          <t>167575609124204</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>I Love Dogs Forge 'N Fetch</t>
+          <t>Brandi’s Southern Doodles &amp; Poodles, LLC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61591593760286</t>
+          <t>https://www.facebook.com/BrandisSouthernDoodlesandPoodles</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dogs, P_dog=1.00)</t>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: poodles, doodles)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>puppy (P=1.00)</t>
+          <t>non_dog (P=0.85)</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>dogs</t>
+          <t>poodles, doodles</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/753954046_122112615273386458_4146374115223244916_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1079x1078&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Ni6iO7UEIhAQ7kNvwEX3aDq&amp;_nc_oc=Adrz8cAAO2KmFnkZuRFza8iqAvdl16K9ANiruVQlW0Gf0J8H84W8375VrlBdRXWu9Uo&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=HP3imHJzQbwK5_D9L5y4YQ&amp;_nc_ss=7b2a8&amp;oh=00_AQO2tZAE_PYlpJU34MDZlFQD15hI23WOU7elgwST5qh6bw&amp;oe=6ADE430D</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/290874043_167575609124204_8051960330153032304_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=YQZymWJ3-y4Q7kNvwHVe2fB&amp;_nc_oc=Adrqjmp_DmhWnTiBimR93_qm4amEiy2QcxlW4LVFWkB4fnSxouhi4zAZCyA3UsGb2NM&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=pelMvMZbxRbN5uMQAHbS1Q&amp;_nc_ss=7b2a8&amp;oh=00_AQO4M9H1q9mWC48B-W7v-25Td6UV0PlCaHWQh7MMjNl9Lg&amp;oe=6ADE4DE9</t>
         </is>
       </c>
     </row>
@@ -753,40 +753,40 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>61594775080228</t>
+          <t>224535483884124</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Yorkshih Pupco</t>
+          <t>Galaxy Golden Retrievers</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61594775080228</t>
+          <t>https://www.facebook.com/galaxygoldenretrievers</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: breeder, breeders, pupco)</t>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: golden retrievers, retrievers)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>non_dog (P=0.95)</t>
+          <t>non_dog (P=0.85)</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>breeder, breeders, pupco, yorkshire, shih tzu, pup, puppy, dog</t>
+          <t>golden retrievers, retrievers, goldens</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/830513831_122102418099492502_4902222354387580447_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx800x800&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=EsJnYIDH-P0Q7kNvwF_S4j8&amp;_nc_oc=AdolxT1vtUo6WEzYifsxx3wdxMH5qMFOkvd3Dv6_4e8LN-DXvU8v0UGTTe9ILvMYdig&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=HP3imHJzQbwK5_D9L5y4YQ&amp;_nc_ss=7b2a8&amp;oh=00_AQMxPuNOASl5lLsgUP07MQPcBGYSzfk1IVucqOeJFMC7Vw&amp;oe=6ADE47B5</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/368381343_224535483884124_7262168979554044494_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx956x960&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Fozk3m8ofZUQ7kNvwHk3Dev&amp;_nc_oc=AdoY_TUW80Ixf2IsE5KV1w5oPOPzi_ptw2OQjkTde9VcAhkPP-WYZF--YAjl8MBH2kY&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=W3-63CRhSeTi0X6tRyjinQ&amp;_nc_ss=7b2a8&amp;oh=00_AQMz1t90gf2bxZRAOPmzS40sKuqK23udRILxoIZ99ekuEA&amp;oe=6ADE565A</t>
         </is>
       </c>
     </row>
@@ -796,40 +796,40 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>61551532070511</t>
+          <t>727311656940554</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Oakhaven Acres Aussies- AKC Australian Shepherds</t>
+          <t>Golden Puppies</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61551532070511</t>
+          <t>https://www.facebook.com/goldenpuppies2004</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: akc, shepherds, aussies)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, puppy, dog)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>non_dog (P=0.95)</t>
+          <t>adult_dog (P=1.00)</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0.95</v>
+        <v>1</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>akc, shepherds, aussies, australian shepherd</t>
+          <t>puppies, puppy, dog, goldens</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/427143042_122133778058051069_7335697382670797595_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1170x1170&amp;_nc_cat=102&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=FXFGb8mH_kEQ7kNvwGyHi8Y&amp;_nc_oc=Adr7QPqn9TWmoPvg5PVMQ0XhE5o0u6TghXQJDLA6BUNVWjNBCwYGYaq3OEn_ED4uQBQ&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=HP3imHJzQbwK5_D9L5y4YQ&amp;_nc_ss=7b2a8&amp;oh=00_AQPI-hF_GlM-ASJS-S_YyieWtSZ-BN8gDQKxOwDEdZiD9Q&amp;oe=6ADE3592</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/530235894_727311656940554_8801302940165924973_n.jpg?stp=c507.540.1422.1423a_cp0_dst-jpg_tt6&amp;cstp=mx1422x1423&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Hoq6NuCogV8Q7kNvwEB7GfP&amp;_nc_oc=AdpXKgkhgvSL0qJc_-82d8oRZNf-J9oCE9OiklOMFQxEb4pDVAiVaMHpK6DlJcTS0zU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=W3-63CRhSeTi0X6tRyjinQ&amp;_nc_ss=7b2a8&amp;oh=00_AQMVJL9PwWeX-QIYDMIBsq4DIFAw8HukSKTfDaAwYbrD_A&amp;oe=6ADE3D7D</t>
         </is>
       </c>
     </row>
@@ -839,40 +839,40 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>61588242310496</t>
+          <t>1713907270555802</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bottom Top Basset’s</t>
+          <t>Beauty and the Beast Shih Tzu</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61588242310496</t>
+          <t>https://www.facebook.com/BeautysShihTzu</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: basset)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: shih tzu, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>non_dog (P=0.85)</t>
+          <t>adult_dog (P=1.00)</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>basset</t>
+          <t>shih tzu</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/825267903_122124942699274743_5172081817443253017_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=2Nx0sQfNEdYQ7kNvwEEHpwQ&amp;_nc_oc=AdrGG7ydqjr2dqoG-wqqKcuIg7HL53ZRvs1rZ-bH9HiCb8i1oCMaFNiwOeeYbo3oF-8&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=d0EBryXU1UgygpoH5zQ81A&amp;_nc_ss=7b2a8&amp;oh=00_AQMClSH_3Pr7Fo8AETARMoZoeLNCTt3jcoMjIHQnaOycgg&amp;oe=6ADE5311</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/854337368_1713907270555802_3166642091340115423_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=WCfvxI38zx8Q7kNvwEjrNu9&amp;_nc_oc=Adob3XQ7o0vsKe8Rgt9BxFxPabxD6XcuUfYHgIvADOzYI7RB2-3hq8lgzeK92i34aLk&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=W3-63CRhSeTi0X6tRyjinQ&amp;_nc_ss=7b2a8&amp;oh=00_AQPuUc2qyLkwN3kVJj2jjdzhdI_z8WbladuDG1hEbwWhcQ&amp;oe=6ADE3F59</t>
         </is>
       </c>
     </row>
@@ -882,27 +882,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>61594781858150</t>
+          <t>122193969698840038</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pawsome Daschund Puppies</t>
+          <t>Shih Tzu Love'r</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61594781858150</t>
+          <t>https://www.facebook.com/shihtzulovers02</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, puppy, dog)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: shih tzu, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>adult_dog (P=1.00)</t>
+          <t>puppy (P=1.00)</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -910,12 +910,12 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>puppies, puppy, dog</t>
+          <t>shih tzu</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/839806917_122108759649492728_2289165301397021762_n.jpg?stp=c0.0.540.540a_cp0_dst-jpg_tt6&amp;cstp=mx540x540&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=2UvAoPM99EEQ7kNvwHxkrkL&amp;_nc_oc=AdrESu6ut2JVf7qtFuvRkFUswJlaQsHriYHFk6b4MTqBZbGWen-GSMMdPRKni2uuexU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=y4c-DeRUU11dMr2UX5j8JA&amp;_nc_ss=7b2a8&amp;oh=00_AQOcoHhyZy0YKhN_sW7QUn2AkPK_Kt9grNoXmvOIjVca6w&amp;oe=6ADE3700</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/751883689_122193969698840038_5392462303461976167_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=6neccbWYohAQ7kNvwE-4Qlt&amp;_nc_oc=AdpFYRDPh9z0v8qmF9i8I8G5BGFYcr52nPHR8mg1--IoueFm2rurFK3muXwEoS5i8Ng&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=W3-63CRhSeTi0X6tRyjinQ&amp;_nc_ss=7b2a8&amp;oh=00_AQMjw30eryhv4uI7o57_txEXm663N77XwQ5uan6uE4rzdw&amp;oe=6ADE3DD7</t>
         </is>
       </c>
     </row>
@@ -925,40 +925,40 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>61594195772352</t>
+          <t>134105013011006</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Jose MiniPuppies</t>
+          <t>Lil’ Bit’s Shih Tzu PUPS of NC</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61594195772352</t>
+          <t>https://www.facebook.com/lilbitspups</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppy, dog)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: pups, shih tzu, puppy)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>puppy (P=1.00)</t>
+          <t>adult_dog (P=1.00)</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.9996</v>
+        <v>1</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>puppy, dog</t>
+          <t>pups, shih tzu, puppy, dog, puppies</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/855646238_122124401871473192_6657591073014986332_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1053x1050&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=fpciUtL0RqgQ7kNvwHvDvml&amp;_nc_oc=AdrkOtpO68tVOeHRBbQwGKPXDMKv6JIvACChqv-71ZDlzMeiB7o2zM5DLwzGe9EmfD0&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=y4c-DeRUU11dMr2UX5j8JA&amp;_nc_ss=7b2a8&amp;oh=00_AQMoTuCS5W_fKqhvV4ISSWCagCN3T9NI57HCSPDhZ-PTug&amp;oe=6ADE44CF</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/349320352_134105013011006_4377198773058659903_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1170x1170&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=dWgF00YllvgQ7kNvwFoblVY&amp;_nc_oc=AdpcjWk8V-ykX3wgyPm0TKbA-DOC6ueNtT7fBoymBY0v1cD56Oc5vKGCFhYxxsgQkeo&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=W3-63CRhSeTi0X6tRyjinQ&amp;_nc_ss=7b2a8&amp;oh=00_AQNoIW2nGko2V6-xIK8cQ1KYCC5mlJGs3kvJHcor3w8_KQ&amp;oe=6ADE4B68</t>
         </is>
       </c>
     </row>
@@ -968,22 +968,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1489668089832323</t>
+          <t>103750072031616</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Tambali Pembroke welsh corgis est. 1998</t>
+          <t>Willow Oak Farm White Labs</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/Tambalicorgis</t>
+          <t>https://www.facebook.com/willowoakfarmwhitelabs</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: corgis, pembroke)</t>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: labs)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -996,12 +996,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>corgis, pembroke</t>
+          <t>labs</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/628787013_1489668089832323_6013872381075739493_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1024x1024&amp;_nc_cat=106&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=78QAEnU19pYQ7kNvwEdF6M8&amp;_nc_oc=AdqAnBQs8chVNgaUNDOr8kq6u2kY2oQbBOhBaUC2ubsjg00tY22Uoqr4BrypC7ogkqs&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=y4c-DeRUU11dMr2UX5j8JA&amp;_nc_ss=7b2a8&amp;oh=00_AQOjodBjmS0_j0jf04e6FFQTcRlWSJdebAz-hS_2oJMDmQ&amp;oe=6ADE43E7</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/239326327_103750072031616_8246519884499016640_n.png?stp=c226.0.1036.1036a_cp0_dst-png&amp;cstp=mx1036x1036&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=VoCMcdQms2kQ7kNvwHGcnao&amp;_nc_oc=Adolgiyk1m5c6zXpxZMofnxHL--Gs1-I-UW6ScqXoisJ0xL8nPGLYLJdAvZFomXgTFM&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=x_eCW6M3_boLIlu9Xz2UVw&amp;_nc_ss=7b2a8&amp;oh=00_AQPnsGKYXLsOnCGlBqyLiHfmVnP-v7OBQ_Wz0737M7M1ug&amp;oe=6ADE538E</t>
         </is>
       </c>
     </row>
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>61591427093472</t>
+          <t>1930354481705111</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Franklineschipperkes Kennel</t>
+          <t>Prairie Creek Kennel</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61591427093472</t>
+          <t>https://www.facebook.com/PrairieCreekKennel</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>adult_dog (P=1.00)</t>
+          <t>puppy (P=1.00)</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/818936768_122125355133380903_6137241591030814058_n.jpg?stp=cp6_dst-jpg_tt6&amp;cstp=mx845x845&amp;_nc_cat=104&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=hekGuXarAzkQ7kNvwHSLKZB&amp;_nc_oc=AdqK_Pk1Vju7cJ78k38AbjiQxUPrgFfqzKFFtHS2yrhswAlzj4zAGl4mSWwr17GgtnE&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=y4c-DeRUU11dMr2UX5j8JA&amp;_nc_ss=7b2a8&amp;oh=00_AQMzIJk4OUXN4yGcWHszoK85mTqgYKndymGkEqsoTNLJQA&amp;oe=6ADE4719</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/787924714_1930354481705111_8023386184839815697_n.jpg?stp=c0.0.1118.1118a_cp0_dst-jpg_tt6&amp;cstp=mx1118x1118&amp;_nc_cat=107&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=QUF7osBv29sQ7kNvwEs5iLa&amp;_nc_oc=AdqzG72wd25ONZrGn15WhiecIpy6h64OKmGOdQAQGnirgeFQKii7WnI_hZJHUtU9xtU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=x_eCW6M3_boLIlu9Xz2UVw&amp;_nc_ss=7b2a8&amp;oh=00_AQN0rHZ7YxrseRLDb_rYSmbJf4O0iMqScL10q5MBAWNd0g&amp;oe=6ADE686E</t>
         </is>
       </c>
     </row>
@@ -1054,27 +1054,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>61593315111061</t>
+          <t>434190195177077</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dachshund Puppies For Adoption And Rehoming</t>
+          <t>Creme of the Crop Dachshunds</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61593315111061</t>
+          <t>https://www.facebook.com/englishcreammniaturedachshunds</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: puppies, dachshund, puppy)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dachshunds, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>puppy (P=1.00)</t>
+          <t>adult_dog (P=1.00)</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -1082,12 +1082,12 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>puppies, dachshund, puppy, dog</t>
+          <t>dachshunds</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/766890471_122093395911443837_496170756872224230_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx828x828&amp;_nc_cat=100&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=ihYNssPKU28Q7kNvwEDZvlm&amp;_nc_oc=AdqfWpLpHPGHmq5J1VKT75IRA-swUUjpIjvWsYT90OxxjutYdMMbhfsCNAn4PNy0MWw&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=te8O4haIQ4bk8DSKcpSW7w&amp;_nc_ss=7b2a8&amp;oh=00_AQPNEnh89ueLb2hAllV42UGJvYLcE2NzbTXbGNnpUNbBcg&amp;oe=6ADE644E</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/277559970_434190195177077_5291667728461596283_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1242x1242&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Af-UHt10BhYQ7kNvwFKMFhu&amp;_nc_oc=Adq4GLGLEcT48PJP2FGuJITIIl12xW0MqVFnpLVN8ykxJJA2HyfIdvsvGCC6h1FU1bc&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=nWISXh2b8NBnOu23IzNfEw&amp;_nc_ss=7b2a8&amp;oh=00_AQM5eU7ropmhOAZJKXeubfTKexBF8l2_bxbDjXlsMd7GCw&amp;oe=6ADE5970</t>
         </is>
       </c>
     </row>
@@ -1097,22 +1097,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>61594494459425</t>
+          <t>122094153387516831</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Autumn's Aussies</t>
+          <t>Salvați cățeii de la Popești-Iași</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61594494459425</t>
+          <t>https://www.facebook.com/SalvatiCateiiDeLaPopesti</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: aussies, australian shepherd, P_dog=1.00)</t>
+          <t>AI Thị giác nhận diện cún con sắc nét (Puppy=0.93, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1123,14 +1123,10 @@
       <c r="G16" t="n">
         <v>1</v>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>aussies, australian shepherd</t>
-        </is>
-      </c>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/820934527_2313498826091469_1498160885209143484_n.jpg?stp=c0.0.1536.1536a_cp0_dst-jpg_tt6&amp;cstp=mx1536x1536&amp;_nc_cat=109&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=L03VojkGVZUQ7kNvwEmEWpp&amp;_nc_oc=AdpipHwllV-m4oMIMNa0_C0eG8SYzQy-oJfiT01OuEgrzjRX2jTN7jORBhtWizMu61Y&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=te8O4haIQ4bk8DSKcpSW7w&amp;_nc_ss=7b2a8&amp;oh=00_AQNfQcVVHLnK9yS2OtyTyFQgwP57d7A1ktjz9h38oZnzCQ&amp;oe=6ADE3FE9</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/847550055_122094153387516831_8056891142274074859_n.jpg?stp=c0.70.1500.1500a_cp0_dst-jpg_tt6&amp;cstp=mx1500x1500&amp;_nc_cat=101&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=nmoR64VsmXUQ7kNvwEu-_DI&amp;_nc_oc=AdomVof3gO20cj8WM2qq8xPDzwL6bA_d9roWWyw4iv-1kmsLcGgfYkQpEnN8p3eD9XU&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=nWISXh2b8NBnOu23IzNfEw&amp;_nc_ss=7b2a8&amp;oh=00_AQPm9thyDGnE8BmYq268iL2SrHXYV6zqXBKFWTM_JFnHew&amp;oe=6ADE44D3</t>
         </is>
       </c>
     </row>
@@ -1140,40 +1136,40 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>122193681896610895</t>
+          <t>1138905091673145</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Knock &amp; Bark Miniature Schnauzer.</t>
+          <t>Hyde Park Cavaliers</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/knockandbark</t>
+          <t>https://www.facebook.com/hyde.park.cavaliers.2025</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: schnauzer, miniature schnauzer, P_dog=0.97)</t>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: cavalier, P_dog=1.00)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>puppy (P=0.97)</t>
+          <t>adult_dog (P=1.00)</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0.9741</v>
+        <v>1</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>schnauzer, miniature schnauzer</t>
+          <t>cavalier</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/779082815_122193681896610895_1254854747032187011_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1134x1122&amp;_nc_cat=105&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=N6pIjA1Ts40Q7kNvwGdzE7P&amp;_nc_oc=AdrKeMKHlIsY0Br3XkfOG2hxdtvMcmsaoRr84NZDJtCAPggWhjKVPK2mvbARdKt8b_A&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=te8O4haIQ4bk8DSKcpSW7w&amp;_nc_ss=7b2a8&amp;oh=00_AQOOfR66vg0y_jnCql9iGHPoPUknemKeAXcUGQCJ5PiMOw&amp;oe=6ADE2F3C</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/552894529_1138905091673145_212893724666853543_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=110&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=tb5968Uum_8Q7kNvwF09BmR&amp;_nc_oc=AdoFUfd1wwWodC1ZSndp48NB8ar3nHcoCGpKz5UNfbs0gWdyTk1cWhfg9G3Y9Oc3Zfg&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=nWISXh2b8NBnOu23IzNfEw&amp;_nc_ss=7b2a8&amp;oh=00_AQPdYZGVKj-ASBzvtzllRKTEsYbVY2rLz1IXMuYvrfXbEA&amp;oe=6ADE3C32</t>
         </is>
       </c>
     </row>
@@ -1183,22 +1179,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>61593913773814</t>
+          <t>122123912342347266</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Responsible Breeder Mentorship Program</t>
+          <t>MiniDox Pups</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/profile.php?id=61593913773814</t>
+          <t>https://www.facebook.com/minidoxpups</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: breeder)</t>
+          <t>B2B Breeder / Chủ trại cún xác thực qua NLP &amp; Chân dung Chủ trại (Breeder: pups, puppy, dog)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1211,12 +1207,141 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>breeder</t>
+          <t>pups, puppy, dog, puppies</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/789960755_10215640356039617_8106197547239706512_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1254x1254&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=Ch42QEEATugQ7kNvwFkzIiS&amp;_nc_oc=Adphq4c8PLfRYPgEWIBtAJ-M8vh4V2BGW3LeogcZpQlX8eo9WjUJSbS0GNyPedmjw2I&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=te8O4haIQ4bk8DSKcpSW7w&amp;_nc_ss=7b2a8&amp;oh=00_AQN5vX4_YYWjLBxPJO8dxEdp3cxECEz9Rb-Q5FKwVbRF9w&amp;oe=6ADE3182</t>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/453383289_122123912342347266_388495722924606013_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx641x640&amp;_nc_cat=103&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=7ES5_0tyRfwQ7kNvwE7D1XU&amp;_nc_oc=AdoJKwODYxrlaVzua3BMEIZXWnPoDGVcIzpl-s17BjcF6334NCCXeGLHf_hoeChYpcE&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=nWISXh2b8NBnOu23IzNfEw&amp;_nc_ss=7b2a8&amp;oh=00_AQM0t8pBAyJVLRiu7WdcIl_F9jMEktziUP3kgcN99WY55Q&amp;oe=6ADE3D47</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>855344712613820</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sausage Dog Central</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/SausageDogCentral</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: dog, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>dog</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/360084077_855344712613820_7250726187422931738_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1843x1843&amp;_nc_cat=1&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=EeI4jy4NI6gQ7kNvwHNXgJh&amp;_nc_oc=AdpYXAV-Q_oPfYJlJdBpYbAYLcOjhJypZZdQXPDMKnE3XUqsK8Gr4KuNdMPajEkKrLI&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=ak9sxYgbexO8hxOyCbHoeQ&amp;_nc_ss=7b2a8&amp;oh=00_AQNA75k3wb8Wp2XBtYPTl7XL18k0_dhj93RTFjv5rqZIPg&amp;oe=6ADE416F</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>4486464461616223</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Montpelier Cavaliers</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/sarah.vasyukhnevich</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Chó xác thực qua Từ khóa &amp; AI (Từ khóa: cavalier, P_dog=1.00)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>adult_dog (P=1.00)</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>cavalier</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/717402555_4486464461616223_2174404301963023400_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx1024x1024&amp;_nc_cat=111&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=t_4vuELx2NgQ7kNvwEsfR7S&amp;_nc_oc=AdoJS_nk0XF_8i8yMCxgNnHJFVKgKbHab_dzSD08etDlPt5Okrznfqq9QVaxxpJxNHY&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=ak9sxYgbexO8hxOyCbHoeQ&amp;_nc_ss=7b2a8&amp;oh=00_AQNVLcpIjOWLRxgCTIh3-VO_YwZYmcWZKEwHU5EL5rq7dw&amp;oe=6ADE55CF</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>25642511325416375</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Aurora Lopez Perez</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/aurora.p.lopez</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Khách hàng nuôi cún xác thực qua NLP &amp; Tên (Từ khóa: shih tzu)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>non_dog (P=0.85)</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>shih tzu</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>https://scontent.fsgn8-4.fna.fbcdn.net/v/t39.30808-1/623396454_25642511325416375_1384894326437316373_n.jpg?stp=cp0_dst-jpg_tt6&amp;cstp=mx960x960&amp;_nc_cat=108&amp;_nc_map=urlgen_bucketless&amp;ccb=1-7&amp;_nc_sid=edd80f&amp;_nc_ohc=G9Z8RlS_0aUQ7kNvwGXFEQU&amp;_nc_oc=Ado2UrFjqY2E7cXSKqd6cutgVKUlenoSP-wHYT7DZleC0eT_7AfJ83Uu7ai1ku8vrwQ&amp;_nc_zt=24&amp;_nc_ht=scontent.fsgn8-4.fna&amp;_nc_gid=ak9sxYgbexO8hxOyCbHoeQ&amp;_nc_ss=7b2a8&amp;oh=00_AQP8MhvOXcjrxB-f1wAOvmpBnhwk01jQzQQHvj7yeFZQcQ&amp;oe=6ADE54B6</t>
         </is>
       </c>
     </row>

</xml_diff>